<commit_message>
Template: add Seller Code (C) + Seller Name (D) columns
</commit_message>
<xml_diff>
--- a/pdtracker/cursive_Trial_Template.xlsx
+++ b/pdtracker/cursive_Trial_Template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,25 +49,6 @@
       <color rgb="000F172A"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -94,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,10 +83,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -513,8 +490,6 @@
           <t>B0G1TN136B</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -527,16 +502,6 @@
           <t>MOBHCQ5GJDRB3DUE</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>RSK01</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Rahul Shopperskart</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -549,12 +514,6 @@
           <t>35295295</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>RSK01</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -567,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -653,79 +612,17 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>NEW COLUMNS (optional — for Buy Box tracking):</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4. Seller Code (Col C, optional) — your internal code (e.g. RSK01) to filter Reports by seller.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>4. Seller Code (Col C, OPTIONAL):</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Your internal code for this seller account (e.g. RSK01).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      If you manage products for multiple sellers, give each a unique code.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Used to filter the Reports per seller.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>5. Seller Name (Col D, OPTIONAL):</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      The EXACT seller name as shown by the marketplace.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Example: "Cursive World Pvt Ltd", "Rahul Shopperskart"</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Required to enable Buy Box Lost tracking for this product.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Leave blank if you don't care about Buy Box tracking — that part is skipped.</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5. Seller Name (Col D, optional) — exact marketplace seller name. Required to enable Buy Box tracking for this product.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Template: clean E + F seller cols (white fill)
</commit_message>
<xml_diff>
--- a/pdtracker/cursive_Trial_Template.xlsx
+++ b/pdtracker/cursive_Trial_Template.xlsx
@@ -937,20 +937,12 @@
       <c r="Z1" s="8" t="n"/>
     </row>
     <row r="2" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
+      <c r="A2" s="9" t="n"/>
       <c r="B2" s="10">
         <f>IF(A2="","",IF(A2="Amazon","ASIN",IF(A2="Flipkart","FSN",IF(A2="Meesho","Product ID",IF(A2="Myntra","Style ID",IF(A2="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>B0B561VFWK</t>
-        </is>
-      </c>
+      <c r="C2" s="12" t="n"/>
       <c r="D2" s="11">
         <f>IF(C2="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -979,20 +971,12 @@
       <c r="Z2" s="8" t="n"/>
     </row>
     <row r="3" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
+      <c r="A3" s="9" t="n"/>
       <c r="B3" s="10">
         <f>IF(A3="","",IF(A3="Amazon","ASIN",IF(A3="Flipkart","FSN",IF(A3="Meesho","Product ID",IF(A3="Myntra","Style ID",IF(A3="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>B0F1MWJV6Z</t>
-        </is>
-      </c>
+      <c r="C3" s="12" t="n"/>
       <c r="D3" s="11">
         <f>IF(C3="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1021,20 +1005,12 @@
       <c r="Z3" s="8" t="n"/>
     </row>
     <row r="4" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
+      <c r="A4" s="9" t="n"/>
       <c r="B4" s="10">
         <f>IF(A4="","",IF(A4="Amazon","ASIN",IF(A4="Flipkart","FSN",IF(A4="Meesho","Product ID",IF(A4="Myntra","Style ID",IF(A4="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>B0D7VW9ZC9</t>
-        </is>
-      </c>
+      <c r="C4" s="12" t="n"/>
       <c r="D4" s="11">
         <f>IF(C4="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1063,20 +1039,12 @@
       <c r="Z4" s="8" t="n"/>
     </row>
     <row r="5" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
+      <c r="A5" s="9" t="n"/>
       <c r="B5" s="10">
         <f>IF(A5="","",IF(A5="Amazon","ASIN",IF(A5="Flipkart","FSN",IF(A5="Meesho","Product ID",IF(A5="Myntra","Style ID",IF(A5="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>B0BCKMZY1V</t>
-        </is>
-      </c>
+      <c r="C5" s="12" t="n"/>
       <c r="D5" s="11">
         <f>IF(C5="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1105,20 +1073,12 @@
       <c r="Z5" s="8" t="n"/>
     </row>
     <row r="6" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
+      <c r="A6" s="9" t="n"/>
       <c r="B6" s="10">
         <f>IF(A6="","",IF(A6="Amazon","ASIN",IF(A6="Flipkart","FSN",IF(A6="Meesho","Product ID",IF(A6="Myntra","Style ID",IF(A6="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>B0G6DVB6DG</t>
-        </is>
-      </c>
+      <c r="C6" s="12" t="n"/>
       <c r="D6" s="11">
         <f>IF(C6="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1147,20 +1107,12 @@
       <c r="Z6" s="8" t="n"/>
     </row>
     <row r="7" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
+      <c r="A7" s="9" t="n"/>
       <c r="B7" s="10">
         <f>IF(A7="","",IF(A7="Amazon","ASIN",IF(A7="Flipkart","FSN",IF(A7="Meesho","Product ID",IF(A7="Myntra","Style ID",IF(A7="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>SMWGEH7WC8F4VKKZ</t>
-        </is>
-      </c>
+      <c r="C7" s="12" t="n"/>
       <c r="D7" s="11">
         <f>IF(C7="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1189,20 +1141,12 @@
       <c r="Z7" s="8" t="n"/>
     </row>
     <row r="8" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
+      <c r="A8" s="9" t="n"/>
       <c r="B8" s="10">
         <f>IF(A8="","",IF(A8="Amazon","ASIN",IF(A8="Flipkart","FSN",IF(A8="Meesho","Product ID",IF(A8="Myntra","Style ID",IF(A8="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>SMWH44GEGTYQHPJ2</t>
-        </is>
-      </c>
+      <c r="C8" s="12" t="n"/>
       <c r="D8" s="11">
         <f>IF(C8="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1231,20 +1175,12 @@
       <c r="Z8" s="8" t="n"/>
     </row>
     <row r="9" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
+      <c r="A9" s="9" t="n"/>
       <c r="B9" s="10">
         <f>IF(A9="","",IF(A9="Amazon","ASIN",IF(A9="Flipkart","FSN",IF(A9="Meesho","Product ID",IF(A9="Myntra","Style ID",IF(A9="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>DUBHDFF7D3JV7ZFY</t>
-        </is>
-      </c>
+      <c r="C9" s="12" t="n"/>
       <c r="D9" s="11">
         <f>IF(C9="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1273,20 +1209,12 @@
       <c r="Z9" s="8" t="n"/>
     </row>
     <row r="10" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
+      <c r="A10" s="9" t="n"/>
       <c r="B10" s="10">
         <f>IF(A10="","",IF(A10="Amazon","ASIN",IF(A10="Flipkart","FSN",IF(A10="Meesho","Product ID",IF(A10="Myntra","Style ID",IF(A10="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>SMWGQHN4RWUTXYMY</t>
-        </is>
-      </c>
+      <c r="C10" s="12" t="n"/>
       <c r="D10" s="11">
         <f>IF(C10="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1315,20 +1243,12 @@
       <c r="Z10" s="8" t="n"/>
     </row>
     <row r="11" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
+      <c r="A11" s="9" t="n"/>
       <c r="B11" s="10">
         <f>IF(A11="","",IF(A11="Amazon","ASIN",IF(A11="Flipkart","FSN",IF(A11="Meesho","Product ID",IF(A11="Myntra","Style ID",IF(A11="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>FLTHC44PVYHFYDQG</t>
-        </is>
-      </c>
+      <c r="C11" s="12" t="n"/>
       <c r="D11" s="11">
         <f>IF(C11="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1357,18 +1277,12 @@
       <c r="Z11" s="8" t="n"/>
     </row>
     <row r="12" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
+      <c r="A12" s="9" t="n"/>
       <c r="B12" s="10">
         <f>IF(A12="","",IF(A12="Amazon","ASIN",IF(A12="Flipkart","FSN",IF(A12="Meesho","Product ID",IF(A12="Myntra","Style ID",IF(A12="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>31666100</v>
-      </c>
+      <c r="C12" s="13" t="n"/>
       <c r="D12" s="11">
         <f>IF(C12="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1397,18 +1311,12 @@
       <c r="Z12" s="8" t="n"/>
     </row>
     <row r="13" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
+      <c r="A13" s="9" t="n"/>
       <c r="B13" s="10">
         <f>IF(A13="","",IF(A13="Amazon","ASIN",IF(A13="Flipkart","FSN",IF(A13="Meesho","Product ID",IF(A13="Myntra","Style ID",IF(A13="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>25542452</v>
-      </c>
+      <c r="C13" s="13" t="n"/>
       <c r="D13" s="11">
         <f>IF(C13="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1437,18 +1345,12 @@
       <c r="Z13" s="8" t="n"/>
     </row>
     <row r="14" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
+      <c r="A14" s="9" t="n"/>
       <c r="B14" s="10">
         <f>IF(A14="","",IF(A14="Amazon","ASIN",IF(A14="Flipkart","FSN",IF(A14="Meesho","Product ID",IF(A14="Myntra","Style ID",IF(A14="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>17668462</v>
-      </c>
+      <c r="C14" s="13" t="n"/>
       <c r="D14" s="11">
         <f>IF(C14="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1477,18 +1379,12 @@
       <c r="Z14" s="8" t="n"/>
     </row>
     <row r="15" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
+      <c r="A15" s="9" t="n"/>
       <c r="B15" s="10">
         <f>IF(A15="","",IF(A15="Amazon","ASIN",IF(A15="Flipkart","FSN",IF(A15="Meesho","Product ID",IF(A15="Myntra","Style ID",IF(A15="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>14035144</v>
-      </c>
+      <c r="C15" s="13" t="n"/>
       <c r="D15" s="11">
         <f>IF(C15="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1517,18 +1413,12 @@
       <c r="Z15" s="8" t="n"/>
     </row>
     <row r="16" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
+      <c r="A16" s="9" t="n"/>
       <c r="B16" s="10">
         <f>IF(A16="","",IF(A16="Amazon","ASIN",IF(A16="Flipkart","FSN",IF(A16="Meesho","Product ID",IF(A16="Myntra","Style ID",IF(A16="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>9162839</v>
-      </c>
+      <c r="C16" s="13" t="n"/>
       <c r="D16" s="11">
         <f>IF(C16="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1557,18 +1447,12 @@
       <c r="Z16" s="8" t="n"/>
     </row>
     <row r="17" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>FirstCry</t>
-        </is>
-      </c>
+      <c r="A17" s="9" t="n"/>
       <c r="B17" s="10">
         <f>IF(A17="","",IF(A17="Amazon","ASIN",IF(A17="Flipkart","FSN",IF(A17="Meesho","Product ID",IF(A17="Myntra","Style ID",IF(A17="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>3391720</v>
-      </c>
+      <c r="C17" s="13" t="n"/>
       <c r="D17" s="11">
         <f>IF(C17="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1597,18 +1481,12 @@
       <c r="Z17" s="8" t="n"/>
     </row>
     <row r="18" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>FirstCry</t>
-        </is>
-      </c>
+      <c r="A18" s="9" t="n"/>
       <c r="B18" s="10">
         <f>IF(A18="","",IF(A18="Amazon","ASIN",IF(A18="Flipkart","FSN",IF(A18="Meesho","Product ID",IF(A18="Myntra","Style ID",IF(A18="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C18" s="13" t="n">
-        <v>16190242</v>
-      </c>
+      <c r="C18" s="13" t="n"/>
       <c r="D18" s="11">
         <f>IF(C18="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1637,18 +1515,12 @@
       <c r="Z18" s="8" t="n"/>
     </row>
     <row r="19" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>FirstCry</t>
-        </is>
-      </c>
+      <c r="A19" s="9" t="n"/>
       <c r="B19" s="10">
         <f>IF(A19="","",IF(A19="Amazon","ASIN",IF(A19="Flipkart","FSN",IF(A19="Meesho","Product ID",IF(A19="Myntra","Style ID",IF(A19="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C19" s="13" t="n">
-        <v>21103392</v>
-      </c>
+      <c r="C19" s="13" t="n"/>
       <c r="D19" s="11">
         <f>IF(C19="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1677,18 +1549,12 @@
       <c r="Z19" s="8" t="n"/>
     </row>
     <row r="20" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>FirstCry</t>
-        </is>
-      </c>
+      <c r="A20" s="9" t="n"/>
       <c r="B20" s="10">
         <f>IF(A20="","",IF(A20="Amazon","ASIN",IF(A20="Flipkart","FSN",IF(A20="Meesho","Product ID",IF(A20="Myntra","Style ID",IF(A20="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C20" s="13" t="n">
-        <v>8225317</v>
-      </c>
+      <c r="C20" s="13" t="n"/>
       <c r="D20" s="11">
         <f>IF(C20="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1717,18 +1583,12 @@
       <c r="Z20" s="8" t="n"/>
     </row>
     <row r="21" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>FirstCry</t>
-        </is>
-      </c>
+      <c r="A21" s="9" t="n"/>
       <c r="B21" s="10">
         <f>IF(A21="","",IF(A21="Amazon","ASIN",IF(A21="Flipkart","FSN",IF(A21="Meesho","Product ID",IF(A21="Myntra","Style ID",IF(A21="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>20471677</v>
-      </c>
+      <c r="C21" s="13" t="n"/>
       <c r="D21" s="11">
         <f>IF(C21="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1757,18 +1617,12 @@
       <c r="Z21" s="8" t="n"/>
     </row>
     <row r="22" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
+      <c r="A22" s="9" t="n"/>
       <c r="B22" s="10">
         <f>IF(A22="","",IF(A22="Amazon","ASIN",IF(A22="Flipkart","FSN",IF(A22="Meesho","Product ID",IF(A22="Myntra","Style ID",IF(A22="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C22" s="13" t="n">
-        <v>44175508</v>
-      </c>
+      <c r="C22" s="13" t="n"/>
       <c r="D22" s="11">
         <f>IF(C22="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1797,18 +1651,12 @@
       <c r="Z22" s="8" t="n"/>
     </row>
     <row r="23" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
+      <c r="A23" s="9" t="n"/>
       <c r="B23" s="10">
         <f>IF(A23="","",IF(A23="Amazon","ASIN",IF(A23="Flipkart","FSN",IF(A23="Meesho","Product ID",IF(A23="Myntra","Style ID",IF(A23="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C23" s="13" t="n">
-        <v>490296740</v>
-      </c>
+      <c r="C23" s="13" t="n"/>
       <c r="D23" s="11">
         <f>IF(C23="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1837,18 +1685,12 @@
       <c r="Z23" s="8" t="n"/>
     </row>
     <row r="24" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
+      <c r="A24" s="9" t="n"/>
       <c r="B24" s="10">
         <f>IF(A24="","",IF(A24="Amazon","ASIN",IF(A24="Flipkart","FSN",IF(A24="Meesho","Product ID",IF(A24="Myntra","Style ID",IF(A24="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C24" s="13" t="n">
-        <v>443545837</v>
-      </c>
+      <c r="C24" s="13" t="n"/>
       <c r="D24" s="11">
         <f>IF(C24="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1877,18 +1719,12 @@
       <c r="Z24" s="8" t="n"/>
     </row>
     <row r="25" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
+      <c r="A25" s="9" t="n"/>
       <c r="B25" s="10">
         <f>IF(A25="","",IF(A25="Amazon","ASIN",IF(A25="Flipkart","FSN",IF(A25="Meesho","Product ID",IF(A25="Myntra","Style ID",IF(A25="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C25" s="13" t="n">
-        <v>521893927</v>
-      </c>
+      <c r="C25" s="13" t="n"/>
       <c r="D25" s="11">
         <f>IF(C25="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>
@@ -1917,18 +1753,12 @@
       <c r="Z25" s="8" t="n"/>
     </row>
     <row r="26" ht="21.95" customHeight="1" thickBot="1">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Meesho</t>
-        </is>
-      </c>
+      <c r="A26" s="9" t="n"/>
       <c r="B26" s="10">
         <f>IF(A26="","",IF(A26="Amazon","ASIN",IF(A26="Flipkart","FSN",IF(A26="Meesho","Product ID",IF(A26="Myntra","Style ID",IF(A26="FirstCry","FC ID",""))))))</f>
         <v/>
       </c>
-      <c r="C26" s="13" t="n">
-        <v>163095016</v>
-      </c>
+      <c r="C26" s="13" t="n"/>
       <c r="D26" s="11">
         <f>IF(C26="","","⚠ Once uploaded, this row cannot be edited. Please double-check Platform and Product ID before uploading.")</f>
         <v/>

</xml_diff>